<commit_message>
Changes in excel file
</commit_message>
<xml_diff>
--- a/src/templates/Voucher_Porting_Template_Nov.xlsx
+++ b/src/templates/Voucher_Porting_Template_Nov.xlsx
@@ -113,7 +113,7 @@
     <t xml:space="preserve">NA</t>
   </si>
   <si>
-    <t xml:space="preserve">STO1008</t>
+    <t xml:space="preserve">STO1009</t>
   </si>
   <si>
     <t xml:space="preserve">AMOUNT PROVIDED FOR OFFICE PARKING RENT ADVANCE FOR THE MONTH OF November 2025 FROM OFIS SPACES PRIVATE LIMITED AGST. BILL/INVOICE NO. OSN2/25-26/01177 DATED 01-NOV-2025 STORES ENTRY / FOLIO NO. - N.A. (RENT EXPENSE) DATED - 01-NOV-2025</t>
@@ -186,7 +186,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -207,6 +207,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -251,8 +256,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -274,12 +283,12 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z11"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="29.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="25"/>
@@ -485,7 +494,7 @@
       <c r="G3" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>30</v>
       </c>
       <c r="I3" s="0" t="s">
@@ -1200,7 +1209,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="29.57"/>

</xml_diff>